<commit_message>
rapport avec capture ecran cas d'erreurs
</commit_message>
<xml_diff>
--- a/data/activity.xlsx
+++ b/data/activity.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K189"/>
+  <dimension ref="A1:K198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10238,6 +10238,476 @@
         </is>
       </c>
     </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-07-16 15:43:19</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>CustomerCreated</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>78945678</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>78945678</t>
+        </is>
+      </c>
+      <c r="F190" t="n">
+        <v>0</v>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>Desktop App</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>Customer user 10 created</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-07-16 15:43:24</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>CustomerCreated</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>12345645</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>12345645</t>
+        </is>
+      </c>
+      <c r="F191" t="n">
+        <v>0</v>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>Marseille</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>Desktop App</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>Customer neyrouz t created</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-07-16 15:43:29</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>CustomerCreated</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>22222222</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>22222222</t>
+        </is>
+      </c>
+      <c r="F192" t="n">
+        <v>0</v>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>Marseille</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>Desktop App</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>Customer maryem created</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-07-16 15:44:26</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Transfer</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>TRX-100074</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>99999999</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>11111111</t>
+        </is>
+      </c>
+      <c r="F193" t="n">
+        <v>100</v>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>Sousse</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>Transfer 99999999 → 11111111</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-07-16 15:44:58</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Transfer</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>TRX-100075</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>77779999</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>91000021</t>
+        </is>
+      </c>
+      <c r="F194" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>Transfer 77779999 → 91000021</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-07-16 15:54:41</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>CustomerCreated</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>78945678</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>78945678</t>
+        </is>
+      </c>
+      <c r="F195" t="n">
+        <v>0</v>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>Desktop App</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>Customer user 10 created</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-07-16 15:56:13</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>CustomerCreated</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>78945678</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>78945678</t>
+        </is>
+      </c>
+      <c r="F196" t="n">
+        <v>0</v>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>Desktop App</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>Customer user 1 created</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-07-16 15:59:34</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Transfer</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>TRX-100076</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>77779999</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>91000021</t>
+        </is>
+      </c>
+      <c r="F197" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>Transfer 77779999 → 91000021</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-07-16 15:59:44</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Transfer</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>TRX-100077</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>77779999</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>91000021</t>
+        </is>
+      </c>
+      <c r="F198" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>Transfer 77779999 → 91000021</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>